<commit_message>
update readme for SA
</commit_message>
<xml_diff>
--- a/ONT-SA/original/historical_sa_recipients_data_dictionary_1969_to_current.xlsx
+++ b/ONT-SA/original/historical_sa_recipients_data_dictionary_1969_to_current.xlsx
@@ -1,10 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10914"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="11_70FC90309CB0043D360ED772F246C157774E4C4B" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BECD1904-297A-5044-A61D-102D613BD75E}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="135" windowWidth="16590" windowHeight="8475"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="18420" windowHeight="24080" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Dictionary" sheetId="1" r:id="rId1"/>
@@ -91,6 +92,9 @@
   <si>
     <t>Total number of social assistance beneficiaries in Ontario 
 The number of beneficiaries refers to the total number of single individuals and heads of family units on social assistance plus all their dependents (i.e., spouses, dependent children and dependent adults).                   na = not available.</t>
+  </si>
+  <si>
+    <t>1969 to current year (yyyy)</t>
   </si>
   <si>
     <r>
@@ -148,26 +152,14 @@
         <rFont val="Arial"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">Data as from April 1998 include recipients of Ontario Works, Ontario Disability Ssuport Program, </t>
+      <t xml:space="preserve">Data as from April 1998 include recipients of Ontario Works, Ontario Disability Ssuport Program, Temporary Care Assistance and Assistance for Children with Severe Disabilities.                                                                                                                                                 </t>
     </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">Temporary Care Assistance and Assistance for Children with Severe Disabilities.                                                                                                                                                 </t>
-    </r>
-  </si>
-  <si>
-    <t>1969 to current year (yyyy)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -250,14 +242,17 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
     </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
   </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -295,7 +290,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -367,7 +362,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -540,18 +535,18 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:D19"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="18.28515625" style="4" customWidth="1"/>
+    <col min="1" max="1" width="18.33203125" style="4" customWidth="1"/>
     <col min="2" max="2" width="56" style="4" customWidth="1"/>
-    <col min="3" max="3" width="57.42578125" style="4" customWidth="1"/>
-    <col min="4" max="4" width="12.28515625" style="4" customWidth="1"/>
-    <col min="5" max="16384" width="8.85546875" style="4"/>
+    <col min="3" max="3" width="57.5" style="4" customWidth="1"/>
+    <col min="4" max="4" width="12.33203125" style="4" customWidth="1"/>
+    <col min="5" max="16384" width="8.83203125" style="4"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" s="1" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
         <v>13</v>
       </c>
@@ -559,13 +554,13 @@
       <c r="C1" s="2"/>
       <c r="D1" s="2"/>
     </row>
-    <row r="2" spans="1:4" s="1" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A2" s="2"/>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
       <c r="D2" s="2"/>
     </row>
-    <row r="3" spans="1:4" s="1" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
         <v>0</v>
       </c>
@@ -579,18 +574,18 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D4" s="4" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A5" s="5" t="s">
         <v>3</v>
       </c>
@@ -601,7 +596,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
       <c r="B6" s="4" t="s">
         <v>16</v>
       </c>
@@ -609,7 +604,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
       <c r="B7" s="4" t="s">
         <v>17</v>
       </c>
@@ -617,7 +612,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
       <c r="B8" s="4" t="s">
         <v>18</v>
       </c>
@@ -625,7 +620,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
       <c r="B9" s="4" t="s">
         <v>19</v>
       </c>
@@ -633,7 +628,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
       <c r="B10" s="4" t="s">
         <v>20</v>
       </c>
@@ -641,7 +636,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
       <c r="B11" s="4" t="s">
         <v>21</v>
       </c>
@@ -649,7 +644,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
       <c r="B12" s="4" t="s">
         <v>22</v>
       </c>
@@ -657,7 +652,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
       <c r="B13" s="4" t="s">
         <v>23</v>
       </c>
@@ -665,7 +660,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
       <c r="B14" s="4" t="s">
         <v>6</v>
       </c>
@@ -673,7 +668,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.2">
       <c r="B15" s="4" t="s">
         <v>7</v>
       </c>
@@ -681,7 +676,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.2">
       <c r="B16" s="4" t="s">
         <v>8</v>
       </c>
@@ -689,7 +684,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="17" spans="1:4" ht="225.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:4" ht="225.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="5" t="s">
         <v>4</v>
       </c>
@@ -697,7 +692,7 @@
         <v>14</v>
       </c>
       <c r="C17" s="7" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D17" s="5" t="s">
         <v>11</v>
@@ -711,7 +706,7 @@
         <v>24</v>
       </c>
       <c r="C18" s="7" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D18" s="5" t="s">
         <v>11</v>

</xml_diff>